<commit_message>
TP finalisé - Acquisition multi-sources
</commit_message>
<xml_diff>
--- a/data/donnees_test.xlsx
+++ b/data/donnees_test.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>50000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="3">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>60000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="4">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>55000</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="5">
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>45000</v>
+        <v>4500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>